<commit_message>
voeg eigen Ubuntu-VM toe aan excel
</commit_message>
<xml_diff>
--- a/SysInfo/system_info.xlsx
+++ b/SysInfo/system_info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,23 @@
       </c>
       <c r="E2" t="n">
         <v>15.73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ubuntu-DevNet-VirtualBox</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>